<commit_message>
changes for feature update
</commit_message>
<xml_diff>
--- a/Document_Catalogue_2026_V1.0.xlsx
+++ b/Document_Catalogue_2026_V1.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\a8ti61\Documents\Document Review Mail\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F494C8B-D265-42E5-B571-0770BCA3A3AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A0F06E2-D823-4805-AB73-C8EE3D962D80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{174F11EF-D037-4CA2-9D13-66BBA84F28A2}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15270" firstSheet="1" activeTab="1" xr2:uid="{174F11EF-D037-4CA2-9D13-66BBA84F28A2}"/>
   </bookViews>
   <sheets>
     <sheet name="Introduction" sheetId="6" r:id="rId1"/>
@@ -106,7 +106,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1260" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1262" uniqueCount="169">
   <si>
     <t>All the documents are to be upto date as per the Review Date</t>
   </si>
@@ -3286,7 +3286,9 @@
       <c r="F11" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="G11" s="47"/>
+      <c r="G11" s="47" t="s">
+        <v>26</v>
+      </c>
       <c r="H11" s="46">
         <v>46157</v>
       </c>
@@ -3321,7 +3323,9 @@
       <c r="F12" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="G12" s="47"/>
+      <c r="G12" s="47" t="s">
+        <v>26</v>
+      </c>
       <c r="H12" s="30">
         <v>43993</v>
       </c>
@@ -14845,15 +14849,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100425AA63552E6DD44A4776F0079EC1931" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f2ca585ec9caaf73760494464ff1028e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5a40e1f1-7edf-47f8-ade6-3fa40173a7ee" xmlns:ns3="90beab9b-5c97-49ef-80e1-8bede52b6c41" xmlns:ns4="921b7353-8eee-4d57-95e7-6707d4aafa1b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c075f32c7e2696fe9b35e4dde31663a7" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="5a40e1f1-7edf-47f8-ade6-3fa40173a7ee"/>
@@ -15113,6 +15108,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -15125,14 +15129,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{088AA5D9-74E2-4846-A9CD-7382D6B424AA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DB55118-D0FF-4B28-B7DA-F08A7996A909}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -15152,6 +15148,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{088AA5D9-74E2-4846-A9CD-7382D6B424AA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C8E337E-A8F4-400E-A781-7137B24692A3}">
   <ds:schemaRefs>

</xml_diff>